<commit_message>
added back missing channel map for bmg read test
</commit_message>
<xml_diff>
--- a/test/inputs/bmg.xlsx
+++ b/test/inputs/bmg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/qr24461/.julia/dev/esm/test/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B918BE8-E07A-7741-80F4-D9A95767F1E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09E0FB2A-C7B2-1B43-915F-CE3652ED8937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17440" activeTab="1" xr2:uid="{7C37CC98-1F4A-4A36-93A3-A48642CDB423}"/>
   </bookViews>
   <sheets>
     <sheet name="Samples" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
   <si>
     <t>Plate</t>
   </si>
@@ -88,6 +88,24 @@
   </si>
   <si>
     <t>BMG</t>
+  </si>
+  <si>
+    <t>ABS_600_0_nm</t>
+  </si>
+  <si>
+    <t>abs600</t>
+  </si>
+  <si>
+    <t>ABS_700_0_nm</t>
+  </si>
+  <si>
+    <t>abs700</t>
+  </si>
+  <si>
+    <t>FI_YFP_pAN1717</t>
+  </si>
+  <si>
+    <t>yfp</t>
   </si>
 </sst>
 </file>
@@ -534,19 +552,42 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DA707B9-0BE9-45E5-A5EE-A3873F0594F1}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>